<commit_message>
Replace recommendation with Critical/High to-confirm line; remove OPEN_ITEMS
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012r6bKnXcJp9a2cyYVk4obL
</commit_message>
<xml_diff>
--- a/skills/contract-review-flagger/templates/Contract_Review_Template.xlsx
+++ b/skills/contract-review-flagger/templates/Contract_Review_Template.xlsx
@@ -609,7 +609,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Produced by the contract review skill from the contract text and the Start2 standards workbook, then checked by a person. Counts and the recommendation update when you edit the Findings sheet.</t>
+          <t>Produced by the contract review skill from the contract text and the Start2 standards workbook, then checked by a person. Counts and the to-confirm line update when you edit the Findings sheet.</t>
         </is>
       </c>
     </row>
@@ -629,7 +629,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Read the role, the counts and the recommendation. Check the role guess first: if it is wrong, nothing else applies.</t>
+          <t>Read the role, the counts and the number of findings to confirm. Check the role guess first: if it is wrong, nothing else applies.</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Do not sign (if already executed, escalate at once). Reject threshold met, hard stop, wrong entity, no liability cap, blank essential fields.</t>
+          <t>Do not sign as it stands. Reject threshold met, hard stop, wrong entity, no liability cap, blank essential fields.</t>
         </is>
       </c>
     </row>
@@ -825,7 +825,7 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Provider, Buyer or Other. The standards cover provider-side contracts only. If the role is not Provider, standards coverage is not applied and the recommendation says so.</t>
+          <t>Provider, Buyer or Other. The standards cover provider-side contracts only. If the role is not Provider, standards coverage is not applied and the To confirm line says so.</t>
         </is>
       </c>
     </row>
@@ -868,12 +868,12 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Recommendation</t>
+          <t>To confirm</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Formula. Draft: any Critical = Escalate; any High = Proceed with named conditions; otherwise Proceed. Executed: no signature gate; Critical items are escalated and High items logged for amendment or renewal.</t>
+          <t>Formula: the number of Critical and High findings. These are logged for a person to confirm; nothing else is recommended.</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>Counts and the recommendation use the Findings sheet only. Coverage severity is a view and is not counted.</t>
+          <t>Counts and the to-confirm line use the Findings sheet only. Coverage severity is a view and is not counted.</t>
         </is>
       </c>
     </row>
@@ -1423,11 +1423,11 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Recommendation</t>
+          <t>To confirm</t>
         </is>
       </c>
       <c r="B19" s="5">
-        <f>IF(OR(B5="",B11=""),"",IF(B11&lt;&gt;"Provider","Not assessed: the standards cover provider-side contracts only",IF(B5="Executed",IF(B15&gt;0,"Executed: escalate Critical items and log High items for amendment or renewal",IF(B16&gt;0,"Executed: log High items for amendment or renewal","Executed: no action required")),IF(B15&gt;0,"Escalate",IF(B16&gt;0,"Proceed with named conditions","Proceed")))))</f>
+        <f>IF(B11="","",IF(B11&lt;&gt;"Provider","Not assessed: the standards cover provider-side contracts only",(B15+B16)&amp;" Critical and High findings to confirm"))</f>
         <v/>
       </c>
       <c r="C19" s="5" t="n"/>

</xml_diff>

<commit_message>
contract-review-flagger: optional term explanations, no rating talk in Issue, no bracket reminder
- Intake asks whether legal terms and clause codes should be explained in plain words
  (summary.explain_terms). When false, plain_language warnings and "Terms used" lines are skipped.
- Issue no longer states or justifies severity, verdict or type; the columns show them. A reason
  for a severity that differs from the rule goes in severity_note, shown as a comment on the
  Severity cell. The validator flags rating talk in Issue and accepts a severity_note in place of
  the old in-text justification.
- Suggested language no longer ends with "Fill the bracketed items before sending."

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DMfeGoX6GYy6toDABTDxog
</commit_message>
<xml_diff>
--- a/skills/contract-review-flagger/templates/Contract_Review_Template.xlsx
+++ b/skills/contract-review-flagger/templates/Contract_Review_Template.xlsx
@@ -1003,7 +1003,7 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Critical, High, Medium or Low (drop-down).</t>
+          <t>Critical, High, Medium or Low (drop-down). A comment on the cell explains a severity that differs from the usual rule.</t>
         </is>
       </c>
     </row>
@@ -1063,7 +1063,7 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>What the clause says in plain words, what it means for Start2 in practice, how it compares with the Start2 standard, and why it has this severity. Low and no-action findings use two sentences.</t>
+          <t>What the clause says in plain words, what it means for Start2 in practice, and how it compares with the Start2 standard. Low and no-action findings use two sentences.</t>
         </is>
       </c>
     </row>
@@ -1087,7 +1087,7 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Wording to propose to the counterparty. For a standard clause, the Start2 standard language with the parties named as in this contract; otherwise wording written for this finding. Fill bracketed items and adjust before sending.</t>
+          <t>Wording to propose to the counterparty. For a standard clause, the Start2 standard language with the parties named as in this contract; otherwise wording written for this finding.</t>
         </is>
       </c>
     </row>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>Where a legal term or a Start2 clause code (for example WARR) is used without explanation, a 'Terms used' line at the end of the cell gives its plain meaning.</t>
+          <t>When plain-language explanations were requested at intake, a legal term or a Start2 clause code (for example WARR) used without explanation gets a 'Terms used' line at the end of the cell giving its plain meaning.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
contract-review-flagger: drop Subjective and Action needed columns; add README
- Findings no longer shows the Subjective and Action needed columns. The subjective and
  action_required flags stay in review.json because they still set severity; the Read Me
  explains both rules.
- README.md describes the whole process, the split between scripts, Claude, the standards and
  the user, the severity rules, how every column on every sheet is computed, and what the
  validator checks.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DMfeGoX6GYy6toDABTDxog
</commit_message>
<xml_diff>
--- a/skills/contract-review-flagger/templates/Contract_Review_Template.xlsx
+++ b/skills/contract-review-flagger/templates/Contract_Review_Template.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents not supplied" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Findings'!$A$1:$K$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Findings'!$A$1:$I$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Coverage'!$A$1:$G$35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Documents not supplied'!$A$1:$H$2</definedName>
   </definedNames>
@@ -576,7 +576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B73"/>
+  <dimension ref="A1:B71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -747,7 +747,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>A finding that needs nothing from Start2 beyond noting it is lowered one severity level and marked No in the Action needed column. Its Action explains why nothing is needed.</t>
+          <t>A finding that needs nothing from Start2 beyond noting it is lowered one severity level. Its Action starts 'No action needed' and says why.</t>
         </is>
       </c>
     </row>
@@ -759,7 +759,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>A finding whose quoted text lets the counterparty alone judge Start2's work, payment or people (for example 'acceptable to Canada', 'to the satisfaction of', 'in its sole discretion') is raised one severity level and marked Yes in the Subjective column.</t>
+          <t>A finding whose quoted text lets the counterparty alone judge Start2's work, payment or people (for example 'acceptable to Canada', 'to the satisfaction of', 'in its sole discretion') is raised one severity level. The judging words are in bold in the Quote.</t>
         </is>
       </c>
     </row>
@@ -1092,332 +1092,308 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>Subjective</t>
-        </is>
-      </c>
-      <c r="B45" s="5" t="inlineStr">
-        <is>
-          <t>Yes when the quoted text lets the counterparty alone judge Start2's work, payment or people. The severity already includes the one-level raise.</t>
-        </is>
-      </c>
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Sheet: Coverage (one row per standard clause)</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>Action needed</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>No when the finding needs nothing beyond noting it. The severity already includes the one-level reduction.</t>
+          <t>Stable clause key from the standards workbook.</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>Sheet: Coverage (one row per standard clause)</t>
-        </is>
-      </c>
-      <c r="B47" s="3" t="n"/>
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Clause</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Clause name.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>Base severity</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>Stable clause key from the standards workbook.</t>
+          <t>Severity if the clause is missing or deviant. Editable for this contract (for example raise anti-bribery to Medium for a government counterparty). n/a for internal rules.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>Clause</t>
+          <t>Verdict</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>Clause name.</t>
+          <t>Conforming, Partial, Deviant, Missing, Not supplied (the contract says the topic is governed by a document that was not supplied), or N/A (drop-down).</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>Base severity</t>
+          <t>Where</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>Severity if the clause is missing or deviant. Editable for this contract (for example raise anti-bribery to Medium for a government counterparty). n/a for internal rules.</t>
+          <t>Contract clause number and page where the clause was found.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>Verdict</t>
+          <t>Severity</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>Conforming, Partial, Deviant, Missing, Not supplied (the contract says the topic is governed by a document that was not supplied), or N/A (drop-down).</t>
+          <t>Formula. Missing, Deviant or Not supplied = Base severity; Partial = one level lower (floor Low); Conforming or N/A = '-'.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>Where</t>
+          <t>Note</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>Contract clause number and page where the clause was found.</t>
+          <t>One line on what is present or absent. Details are in Findings.</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="4" t="inlineStr">
-        <is>
-          <t>Severity</t>
-        </is>
-      </c>
-      <c r="B53" s="5" t="inlineStr">
-        <is>
-          <t>Formula. Missing, Deviant or Not supplied = Base severity; Partial = one level lower (floor Low); Conforming or N/A = '-'.</t>
-        </is>
-      </c>
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Sheet: Checks (one row per execution check)</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>Note</t>
+          <t>#</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>One line on what is present or absent. Details are in Findings.</t>
+          <t>Number of the check in the standards workbook.</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>Sheet: Checks (one row per execution check)</t>
-        </is>
-      </c>
-      <c r="B55" s="3" t="n"/>
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>What is verified before a draft leaves Start2 and again before signature.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>#</t>
+          <t>Result</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>Number of the check in the standards workbook.</t>
+          <t>Pass, Fail, N/A or Cannot verify (drop-down).</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>Check</t>
+          <t>Evidence</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>What is verified before a draft leaves Start2 and again before signature.</t>
+          <t>What was seen, with page references.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>Result</t>
+          <t>Clauses to correct</t>
         </is>
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>Pass, Fail, N/A or Cannot verify (drop-down).</t>
+          <t>For a failed check, each contract clause or page that needs correcting and what to change, numbered.</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="4" t="inlineStr">
-        <is>
-          <t>Evidence</t>
-        </is>
-      </c>
-      <c r="B59" s="5" t="inlineStr">
-        <is>
-          <t>What was seen, with page references.</t>
-        </is>
-      </c>
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Sheet: Documents not supplied (one row per document)</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>Clauses to correct</t>
+          <t>Document</t>
         </is>
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>For a failed check, each contract clause or page that needs correcting and what to change, numbered.</t>
+          <t>The document as the contract names it, with version or date if given.</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="inlineStr">
-        <is>
-          <t>Sheet: Documents not supplied (one row per document)</t>
-        </is>
-      </c>
-      <c r="B61" s="3" t="n"/>
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>Referenced at</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>Every contract clause and page where the document is named, numbered.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>Document</t>
+          <t>Quotes</t>
         </is>
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>The document as the contract names it, with version or date if given.</t>
+          <t>The contract text at each of those places, numbered to match, with the document's name in bold.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>Referenced at</t>
+          <t>Part of contract</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>Every contract clause and page where the document is named, numbered.</t>
+          <t>Yes when the contract says the document applies to or forms part of the contract. Those also appear in Findings as type Not supplied.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>Quotes</t>
+          <t>Governs</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>The contract text at each of those places, numbered to match, with the document's name in bold.</t>
+          <t>What the contract says or shows the document covers. Never a guess at its content.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>Part of contract</t>
+          <t>Effect on this review</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>Yes when the contract says the document applies to or forms part of the contract. Those also appear in Findings as type Not supplied.</t>
+          <t>Which findings and coverage rows could not be completed without it.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>Governs</t>
+          <t>Action</t>
         </is>
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>What the contract says or shows the document covers. Never a guess at its content.</t>
+          <t>How to obtain it and what to check once it is in hand.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>Effect on this review</t>
+          <t>Terms used</t>
         </is>
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>Which findings and coverage rows could not be completed without it.</t>
+          <t>When plain-language explanations were requested at intake, a legal term or a Start2 clause code (for example WARR) used without explanation gets a 'Terms used' line at the end of the cell giving its plain meaning.</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="4" t="inlineStr">
-        <is>
-          <t>Action</t>
-        </is>
-      </c>
-      <c r="B68" s="5" t="inlineStr">
-        <is>
-          <t>How to obtain it and what to check once it is in hand.</t>
-        </is>
-      </c>
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Rules</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>Terms used</t>
+          <t>Counts</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>When plain-language explanations were requested at intake, a legal term or a Start2 clause code (for example WARR) used without explanation gets a 'Terms used' line at the end of the cell giving its plain meaning.</t>
+          <t>Counts and the to-confirm line use the Findings sheet only. Coverage severity is a view and is not counted.</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="inlineStr">
-        <is>
-          <t>Rules</t>
-        </is>
-      </c>
-      <c r="B70" s="3" t="n"/>
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t>Role and intake</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>Before the review, the skill sends one intake message asking the requester to confirm the Start2 entity and role, send any documents the contract names but that were not supplied, and state the purpose. It does not stop again after that.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>Counts</t>
+          <t>Not legal advice</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr">
-        <is>
-          <t>Counts and the to-confirm line use the Findings sheet only. Coverage severity is a view and is not counted.</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="4" t="inlineStr">
-        <is>
-          <t>Role and intake</t>
-        </is>
-      </c>
-      <c r="B72" s="5" t="inlineStr">
-        <is>
-          <t>Before the review, the skill sends one intake message asking the requester to confirm the Start2 entity and role, send any documents the contract names but that were not supplied, and state the purpose. It does not stop again after that.</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="4" t="inlineStr">
-        <is>
-          <t>Not legal advice</t>
-        </is>
-      </c>
-      <c r="B73" s="5" t="inlineStr">
         <is>
           <t>A screen against Start2 standards. Decisions follow the sign-off chain.</t>
         </is>
@@ -1427,12 +1403,12 @@
   <mergeCells count="9">
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A59:B59"/>
+    <mergeCell ref="A68:B68"/>
     <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="A45:B45"/>
     <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A70:B70"/>
-    <mergeCell ref="A61:B61"/>
-    <mergeCell ref="A55:B55"/>
+    <mergeCell ref="A53:B53"/>
     <mergeCell ref="A35:B35"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1744,7 +1720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1756,8 +1732,6 @@
     <col width="70" customWidth="1" min="7" max="7"/>
     <col width="55" customWidth="1" min="8" max="8"/>
     <col width="60" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1806,19 +1780,9 @@
           <t>Suggested language</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Subjective</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Action needed</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K2"/>
+  <autoFilter ref="A1:I2"/>
   <conditionalFormatting sqref="B2:B300">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Critical"</formula>
@@ -1833,18 +1797,12 @@
       <formula>"Low"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
+  <dataValidations count="2">
     <dataValidation sqref="B2:B300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
     <dataValidation sqref="C2:C300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Missing,Partial,Deviant,Client: Reject,Client: Escalate,Client: Conditional,Client: Accept,Unclassified clause,Commercial,Execution,Not supplied,Other"</formula1>
-    </dataValidation>
-    <dataValidation sqref="J2:J300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Yes"</formula1>
-    </dataValidation>
-    <dataValidation sqref="K2:K300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>